<commit_message>
minor edits for clarity
</commit_message>
<xml_diff>
--- a/data/aurignacian-periods.xlsx
+++ b/data/aurignacian-periods.xlsx
@@ -34,13 +34,13 @@
     <t>Aur-P1 (Proto/Early)</t>
   </si>
   <si>
-    <t>43 - 37</t>
+    <t>43 - 37.8</t>
   </si>
   <si>
     <t>Aur-P2 (Evolved/Late)</t>
   </si>
   <si>
-    <t>37 - 32</t>
+    <t>37.8 - 32</t>
   </si>
   <si>
     <t>GI 8 - 6</t>

</xml_diff>